<commit_message>
refactor: update BulkUploadModal styling
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_image_subjective_upload.xlsx
+++ b/frontend/public/templates/sample_image_subjective_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,11 @@
           <t>Observe the industry trend in scenario 1 and provide a summary.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_1.png</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>The trend indicates a shift towards sustainable practices in the 1 sector...</t>
@@ -543,7 +547,11 @@
           <t>Observe the industry trend in scenario 2 and provide a summary.</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_2.png</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>The trend indicates a shift towards sustainable practices in the 2 sector...</t>
@@ -574,7 +582,11 @@
           <t>Observe the industry trend in scenario 3 and provide a summary.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_3.png</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>The trend indicates a shift towards sustainable practices in the 3 sector...</t>
@@ -605,7 +617,11 @@
           <t>Observe the industry trend in scenario 4 and provide a summary.</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_4.png</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>The trend indicates a shift towards sustainable practices in the 4 sector...</t>
@@ -636,7 +652,11 @@
           <t>Observe the industry trend in scenario 5 and provide a summary.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>data_chart_5.png</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>The trend indicates a shift towards sustainable practices in the 5 sector...</t>

</xml_diff>